<commit_message>
refactor defuzzification, fuzzyLogic, fuzzyRules
</commit_message>
<xml_diff>
--- a/peringkat.xlsx
+++ b/peringkat.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -442,32 +442,22 @@
           <t>Score</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Rekomendasi</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="C2" t="n">
-        <v>77</v>
+        <v>30</v>
       </c>
       <c r="D2" t="n">
-        <v>22825</v>
+        <v>45791</v>
       </c>
       <c r="E2" t="n">
-        <v>90</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>tinggi</t>
-        </is>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -475,21 +465,16 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="C3" t="n">
-        <v>73</v>
+        <v>34</v>
       </c>
       <c r="D3" t="n">
-        <v>24704</v>
+        <v>51772</v>
       </c>
       <c r="E3" t="n">
-        <v>90</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>tinggi</t>
-        </is>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -497,21 +482,16 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>66</v>
+        <v>5</v>
       </c>
       <c r="C4" t="n">
-        <v>80</v>
+        <v>12</v>
       </c>
       <c r="D4" t="n">
-        <v>20052</v>
+        <v>26321</v>
       </c>
       <c r="E4" t="n">
-        <v>90</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>tinggi</t>
-        </is>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -519,21 +499,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>69</v>
+        <v>6</v>
       </c>
       <c r="C5" t="n">
-        <v>85</v>
+        <v>27</v>
       </c>
       <c r="D5" t="n">
-        <v>24551</v>
+        <v>50323</v>
       </c>
       <c r="E5" t="n">
-        <v>90</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>tinggi</t>
-        </is>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -541,21 +516,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>78</v>
+        <v>8</v>
       </c>
       <c r="C6" t="n">
-        <v>86</v>
+        <v>42</v>
       </c>
       <c r="D6" t="n">
-        <v>27315</v>
+        <v>54926</v>
       </c>
       <c r="E6" t="n">
-        <v>90</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>tinggi</t>
-        </is>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>